<commit_message>
Full NJSBCL rescrape — both series through 2026-09-20
Both league stages are now complete: Division 1 at 400 matches, Weekenders
Cup at 799.

Widens the Weekenders scrape to cover Group B's top 8, who had no scorecard
data at all — VRK's knockout field is drawn from Group A plus Group B, so
those teams' pages would otherwise have come up empty. Scope is now Group A
+ Group D (league opponents) + Group B's top 8, 580 of the 800 matches.

Skill doc updated with the new scope and three operational gotchas hit this
run: Downloads filename collisions silently copying a stale file, the 45s
CDP timeout on long fetch batches, and Cloudflare tripping at ~420
cumulative fetches.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AJNc76ZNRMV6tmUr3hcWEA
</commit_message>
<xml_diff>
--- a/NJSBCL/data/division1_schedule.xlsx
+++ b/NJSBCL/data/division1_schedule.xlsx
@@ -323,7 +323,7 @@
       </c>
       <c t="inlineStr" r="E3">
         <is>
-          <t xml:space="preserve">08/29/2026</t>
+          <t xml:space="preserve">09/20/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F3">
@@ -333,22 +333,22 @@
       </c>
       <c t="inlineStr" r="G3">
         <is>
-          <t xml:space="preserve">Pway Lions</t>
+          <t xml:space="preserve">Team Highlanders</t>
         </is>
       </c>
       <c t="inlineStr" r="H3">
         <is>
-          <t xml:space="preserve">Parsippany Phoenix XI</t>
+          <t xml:space="preserve">Blue Aces CC</t>
         </is>
       </c>
       <c t="inlineStr" r="I3">
         <is>
-          <t xml:space="preserve">Pway Lions</t>
+          <t xml:space="preserve">Blue Aces CC</t>
         </is>
       </c>
       <c t="inlineStr" r="J3">
         <is>
-          <t xml:space="preserve">Rowdy Rebels</t>
+          <t xml:space="preserve">Plainsboro Knights</t>
         </is>
       </c>
     </row>
@@ -368,7 +368,7 @@
       </c>
       <c t="inlineStr" r="E4">
         <is>
-          <t xml:space="preserve">08/29/2026</t>
+          <t xml:space="preserve">09/20/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F4">
@@ -378,22 +378,22 @@
       </c>
       <c t="inlineStr" r="G4">
         <is>
-          <t xml:space="preserve">Gujarat United XI</t>
+          <t xml:space="preserve">Samudhra Gladiators</t>
         </is>
       </c>
       <c t="inlineStr" r="H4">
         <is>
-          <t xml:space="preserve">Nj Stars CC</t>
+          <t xml:space="preserve">Maha CC</t>
         </is>
       </c>
       <c t="inlineStr" r="I4">
         <is>
-          <t xml:space="preserve">Gujarat United XI</t>
+          <t xml:space="preserve">Maha CC</t>
         </is>
       </c>
       <c t="inlineStr" r="J4">
         <is>
-          <t xml:space="preserve">11spartans</t>
+          <t xml:space="preserve">Mercer Challengers</t>
         </is>
       </c>
     </row>
@@ -413,7 +413,7 @@
       </c>
       <c t="inlineStr" r="E5">
         <is>
-          <t xml:space="preserve">08/29/2026</t>
+          <t xml:space="preserve">09/20/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F5">
@@ -423,22 +423,22 @@
       </c>
       <c t="inlineStr" r="G5">
         <is>
-          <t xml:space="preserve">Newport CC</t>
+          <t xml:space="preserve">Gcc</t>
         </is>
       </c>
       <c t="inlineStr" r="H5">
         <is>
-          <t xml:space="preserve">Aryans</t>
+          <t xml:space="preserve">Fdu Giants</t>
         </is>
       </c>
       <c t="inlineStr" r="I5">
         <is>
-          <t xml:space="preserve">Newport CC</t>
+          <t xml:space="preserve">FDU Giants</t>
         </is>
       </c>
       <c t="inlineStr" r="J5">
         <is>
-          <t xml:space="preserve">Gryffindors</t>
+          <t xml:space="preserve">Storm Riders</t>
         </is>
       </c>
     </row>
@@ -458,7 +458,7 @@
       </c>
       <c t="inlineStr" r="E6">
         <is>
-          <t xml:space="preserve">08/29/2026</t>
+          <t xml:space="preserve">09/20/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F6">
@@ -468,22 +468,22 @@
       </c>
       <c t="inlineStr" r="G6">
         <is>
-          <t xml:space="preserve">Storm Riders</t>
+          <t xml:space="preserve">Desi Warriors</t>
         </is>
       </c>
       <c t="inlineStr" r="H6">
         <is>
-          <t xml:space="preserve">WCC</t>
+          <t xml:space="preserve">Juggernaut</t>
         </is>
       </c>
       <c t="inlineStr" r="I6">
         <is>
-          <t xml:space="preserve">Storm Riders</t>
+          <t xml:space="preserve">Juggernaut</t>
         </is>
       </c>
       <c t="inlineStr" r="J6">
         <is>
-          <t xml:space="preserve">Piscataway Avengers</t>
+          <t xml:space="preserve">Newport CC</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,7 @@
       </c>
       <c t="inlineStr" r="E7">
         <is>
-          <t xml:space="preserve">08/29/2026</t>
+          <t xml:space="preserve">09/20/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F7">
@@ -513,22 +513,22 @@
       </c>
       <c t="inlineStr" r="G7">
         <is>
-          <t xml:space="preserve">Mercer Challengers</t>
+          <t xml:space="preserve">Sreeshti</t>
         </is>
       </c>
       <c t="inlineStr" r="H7">
         <is>
-          <t xml:space="preserve">Plainsboro Eagles</t>
+          <t xml:space="preserve">F5</t>
         </is>
       </c>
       <c t="inlineStr" r="I7">
         <is>
-          <t xml:space="preserve">Mercer Challengers</t>
+          <t xml:space="preserve">F5</t>
         </is>
       </c>
       <c t="inlineStr" r="J7">
         <is>
-          <t xml:space="preserve">F5</t>
+          <t xml:space="preserve">Gujarat United XI</t>
         </is>
       </c>
     </row>
@@ -548,7 +548,7 @@
       </c>
       <c t="inlineStr" r="E8">
         <is>
-          <t xml:space="preserve">08/29/2026</t>
+          <t xml:space="preserve">09/20/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F8">
@@ -558,22 +558,22 @@
       </c>
       <c t="inlineStr" r="G8">
         <is>
-          <t xml:space="preserve">Plainsboro Knights</t>
+          <t xml:space="preserve">Hudson Hurricanes</t>
         </is>
       </c>
       <c t="inlineStr" r="H8">
         <is>
-          <t xml:space="preserve">Jetha 11</t>
+          <t xml:space="preserve">Piscataway Avengers</t>
         </is>
       </c>
       <c t="inlineStr" r="I8">
         <is>
-          <t xml:space="preserve">Plainsboro Knights</t>
+          <t xml:space="preserve">Piscataway Avengers</t>
         </is>
       </c>
       <c t="inlineStr" r="J8">
         <is>
-          <t xml:space="preserve">Juggernaut</t>
+          <t xml:space="preserve">Pway Lions</t>
         </is>
       </c>
     </row>
@@ -593,7 +593,7 @@
       </c>
       <c t="inlineStr" r="E9">
         <is>
-          <t xml:space="preserve">08/29/2026</t>
+          <t xml:space="preserve">09/20/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F9">
@@ -603,22 +603,22 @@
       </c>
       <c t="inlineStr" r="G9">
         <is>
-          <t xml:space="preserve">Jersey Titans</t>
+          <t xml:space="preserve">Falcons</t>
         </is>
       </c>
       <c t="inlineStr" r="H9">
         <is>
-          <t xml:space="preserve">Nj Tigers</t>
+          <t xml:space="preserve">Gryffindors</t>
         </is>
       </c>
       <c t="inlineStr" r="I9">
         <is>
-          <t xml:space="preserve">Jersey Titans</t>
+          <t xml:space="preserve">Gryffindors</t>
         </is>
       </c>
       <c t="inlineStr" r="J9">
         <is>
-          <t xml:space="preserve">Fdu Giants</t>
+          <t xml:space="preserve">PUNJAB XI</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c t="inlineStr" r="E10">
         <is>
-          <t xml:space="preserve">08/29/2026</t>
+          <t xml:space="preserve">09/20/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F10">
@@ -648,22 +648,22 @@
       </c>
       <c t="inlineStr" r="G10">
         <is>
-          <t xml:space="preserve">Nj Braves</t>
+          <t xml:space="preserve">Warriors</t>
         </is>
       </c>
       <c t="inlineStr" r="H10">
         <is>
-          <t xml:space="preserve">Jersey Boys</t>
+          <t xml:space="preserve">11spartans</t>
         </is>
       </c>
       <c t="inlineStr" r="I10">
         <is>
-          <t xml:space="preserve">NJ Braves</t>
+          <t xml:space="preserve">11Spartans</t>
         </is>
       </c>
       <c t="inlineStr" r="J10">
         <is>
-          <t xml:space="preserve">Maha CC</t>
+          <t xml:space="preserve">Blasters</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c t="inlineStr" r="E11">
         <is>
-          <t xml:space="preserve">08/29/2026</t>
+          <t xml:space="preserve">09/20/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F11">
@@ -693,22 +693,22 @@
       </c>
       <c t="inlineStr" r="G11">
         <is>
-          <t xml:space="preserve">Blasters</t>
+          <t xml:space="preserve">Youth For Sewa</t>
         </is>
       </c>
       <c t="inlineStr" r="H11">
         <is>
-          <t xml:space="preserve">Veerans</t>
+          <t xml:space="preserve">Rowdy Rebels</t>
         </is>
       </c>
       <c t="inlineStr" r="I11">
         <is>
-          <t xml:space="preserve">Blasters</t>
+          <t xml:space="preserve">Rowdy Rebels</t>
         </is>
       </c>
       <c t="inlineStr" r="J11">
         <is>
-          <t xml:space="preserve">Blue Aces CC</t>
+          <t xml:space="preserve">Nj Braves</t>
         </is>
       </c>
     </row>
@@ -728,7 +728,7 @@
       </c>
       <c t="inlineStr" r="E12">
         <is>
-          <t xml:space="preserve">08/29/2026</t>
+          <t xml:space="preserve">09/20/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F12">
@@ -738,22 +738,22 @@
       </c>
       <c t="inlineStr" r="G12">
         <is>
-          <t xml:space="preserve">PUNJAB XI</t>
+          <t xml:space="preserve">RHG</t>
         </is>
       </c>
       <c t="inlineStr" r="H12">
         <is>
-          <t xml:space="preserve">Edison Rebelz</t>
+          <t xml:space="preserve">SAMP XI</t>
         </is>
       </c>
       <c t="inlineStr" r="I12">
         <is>
-          <t xml:space="preserve">Punjab XI</t>
+          <t xml:space="preserve">Samp XI</t>
         </is>
       </c>
       <c t="inlineStr" r="J12">
         <is>
-          <t xml:space="preserve">SAMP XI</t>
+          <t xml:space="preserve">Jersey Titans</t>
         </is>
       </c>
     </row>
@@ -773,7 +773,7 @@
       </c>
       <c t="inlineStr" r="E13">
         <is>
-          <t xml:space="preserve">08/30/2026</t>
+          <t xml:space="preserve">09/19/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F13">
@@ -783,22 +783,22 @@
       </c>
       <c t="inlineStr" r="G13">
         <is>
-          <t xml:space="preserve">Team Highlanders</t>
+          <t xml:space="preserve">PUNJAB XI</t>
         </is>
       </c>
       <c t="inlineStr" r="H13">
         <is>
+          <t xml:space="preserve">Nj Stars CC</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="I13">
+        <is>
+          <t xml:space="preserve">Punjab XI</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="J13">
+        <is>
           <t xml:space="preserve">Rowdy Rebels</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="I13">
-        <is>
-          <t xml:space="preserve">Rowdy Rebels</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="J13">
-        <is>
-          <t xml:space="preserve">Jersey Titans</t>
         </is>
       </c>
     </row>
@@ -818,7 +818,7 @@
       </c>
       <c t="inlineStr" r="E14">
         <is>
-          <t xml:space="preserve">08/30/2026</t>
+          <t xml:space="preserve">09/19/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F14">
@@ -828,22 +828,22 @@
       </c>
       <c t="inlineStr" r="G14">
         <is>
-          <t xml:space="preserve">Samudhra Gladiators</t>
+          <t xml:space="preserve">Blasters</t>
         </is>
       </c>
       <c t="inlineStr" r="H14">
         <is>
+          <t xml:space="preserve">Parsippany Phoenix XI</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="I14">
+        <is>
+          <t xml:space="preserve">Blasters</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="J14">
+        <is>
           <t xml:space="preserve">SAMP XI</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="I14">
-        <is>
-          <t xml:space="preserve">Samp XI</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="J14">
-        <is>
-          <t xml:space="preserve">Plainsboro Knights</t>
         </is>
       </c>
     </row>
@@ -863,7 +863,7 @@
       </c>
       <c t="inlineStr" r="E15">
         <is>
-          <t xml:space="preserve">08/30/2026</t>
+          <t xml:space="preserve">09/19/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F15">
@@ -873,22 +873,27 @@
       </c>
       <c t="inlineStr" r="G15">
         <is>
-          <t xml:space="preserve">Gcc</t>
+          <t xml:space="preserve">Nj Braves</t>
         </is>
       </c>
       <c t="inlineStr" r="H15">
         <is>
+          <t xml:space="preserve">Edison Rebelz</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="I15">
+        <is>
+          <t xml:space="preserve">NJ Braves</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="J15">
+        <is>
           <t xml:space="preserve">Blue Aces CC</t>
         </is>
       </c>
-      <c t="inlineStr" r="I15">
+      <c t="inlineStr" r="K15">
         <is>
           <t xml:space="preserve">Blue Aces CC</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="J15">
-        <is>
-          <t xml:space="preserve">Mercer Challengers</t>
         </is>
       </c>
     </row>
@@ -908,7 +913,7 @@
       </c>
       <c t="inlineStr" r="E16">
         <is>
-          <t xml:space="preserve">08/30/2026</t>
+          <t xml:space="preserve">09/19/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F16">
@@ -918,22 +923,22 @@
       </c>
       <c t="inlineStr" r="G16">
         <is>
-          <t xml:space="preserve">Desi Warriors</t>
+          <t xml:space="preserve">Jersey Titans</t>
         </is>
       </c>
       <c t="inlineStr" r="H16">
         <is>
+          <t xml:space="preserve">Veerans</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="I16">
+        <is>
+          <t xml:space="preserve">Jersey Titans</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="J16">
+        <is>
           <t xml:space="preserve">Maha CC</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="I16">
-        <is>
-          <t xml:space="preserve">Maha CC</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="J16">
-        <is>
-          <t xml:space="preserve">Storm Riders</t>
         </is>
       </c>
     </row>
@@ -953,7 +958,7 @@
       </c>
       <c t="inlineStr" r="E17">
         <is>
-          <t xml:space="preserve">08/30/2026</t>
+          <t xml:space="preserve">09/19/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F17">
@@ -963,22 +968,22 @@
       </c>
       <c t="inlineStr" r="G17">
         <is>
-          <t xml:space="preserve">Sreeshti</t>
+          <t xml:space="preserve">Plainsboro Knights</t>
         </is>
       </c>
       <c t="inlineStr" r="H17">
         <is>
+          <t xml:space="preserve">Jersey Boys</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="I17">
+        <is>
+          <t xml:space="preserve">Plainsboro Knights</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="J17">
+        <is>
           <t xml:space="preserve">Fdu Giants</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="I17">
-        <is>
-          <t xml:space="preserve">FDU Giants</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="J17">
-        <is>
-          <t xml:space="preserve">Newport CC</t>
         </is>
       </c>
     </row>
@@ -998,7 +1003,7 @@
       </c>
       <c t="inlineStr" r="E18">
         <is>
-          <t xml:space="preserve">08/30/2026</t>
+          <t xml:space="preserve">09/19/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F18">
@@ -1008,22 +1013,22 @@
       </c>
       <c t="inlineStr" r="G18">
         <is>
-          <t xml:space="preserve">Hudson Hurricanes</t>
+          <t xml:space="preserve">Mercer Challengers</t>
         </is>
       </c>
       <c t="inlineStr" r="H18">
         <is>
+          <t xml:space="preserve">Nj Tigers</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="I18">
+        <is>
+          <t xml:space="preserve">Mercer Challengers</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="J18">
+        <is>
           <t xml:space="preserve">Juggernaut</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="I18">
-        <is>
-          <t xml:space="preserve">Juggernaut</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="J18">
-        <is>
-          <t xml:space="preserve">Gujarat United XI</t>
         </is>
       </c>
     </row>
@@ -1043,7 +1048,7 @@
       </c>
       <c t="inlineStr" r="E19">
         <is>
-          <t xml:space="preserve">08/30/2026</t>
+          <t xml:space="preserve">09/19/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F19">
@@ -1053,22 +1058,22 @@
       </c>
       <c t="inlineStr" r="G19">
         <is>
-          <t xml:space="preserve">Falcons</t>
+          <t xml:space="preserve">Storm Riders</t>
         </is>
       </c>
       <c t="inlineStr" r="H19">
         <is>
+          <t xml:space="preserve">Jetha 11</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="I19">
+        <is>
+          <t xml:space="preserve">Storm Riders</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="J19">
+        <is>
           <t xml:space="preserve">F5</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="I19">
-        <is>
-          <t xml:space="preserve">F5</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="J19">
-        <is>
-          <t xml:space="preserve">Pway Lions</t>
         </is>
       </c>
     </row>
@@ -1088,7 +1093,7 @@
       </c>
       <c t="inlineStr" r="E20">
         <is>
-          <t xml:space="preserve">08/30/2026</t>
+          <t xml:space="preserve">09/19/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F20">
@@ -1098,22 +1103,22 @@
       </c>
       <c t="inlineStr" r="G20">
         <is>
-          <t xml:space="preserve">Warriors</t>
+          <t xml:space="preserve">Newport CC</t>
         </is>
       </c>
       <c t="inlineStr" r="H20">
         <is>
+          <t xml:space="preserve">Plainsboro Eagles</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="I20">
+        <is>
+          <t xml:space="preserve">Newport CC</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="J20">
+        <is>
           <t xml:space="preserve">Piscataway Avengers</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="I20">
-        <is>
-          <t xml:space="preserve">Piscataway Avengers</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="J20">
-        <is>
-          <t xml:space="preserve">PUNJAB XI</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1138,7 @@
       </c>
       <c t="inlineStr" r="E21">
         <is>
-          <t xml:space="preserve">08/30/2026</t>
+          <t xml:space="preserve">09/19/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F21">
@@ -1143,22 +1148,22 @@
       </c>
       <c t="inlineStr" r="G21">
         <is>
-          <t xml:space="preserve">Youth For Sewa</t>
+          <t xml:space="preserve">Gujarat United XI</t>
         </is>
       </c>
       <c t="inlineStr" r="H21">
         <is>
+          <t xml:space="preserve">WCC</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="I21">
+        <is>
+          <t xml:space="preserve">Gujarat United XI</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="J21">
+        <is>
           <t xml:space="preserve">Gryffindors</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="I21">
-        <is>
-          <t xml:space="preserve">Gryffindors</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="J21">
-        <is>
-          <t xml:space="preserve">Blasters</t>
         </is>
       </c>
     </row>
@@ -1178,7 +1183,7 @@
       </c>
       <c t="inlineStr" r="E22">
         <is>
-          <t xml:space="preserve">08/30/2026</t>
+          <t xml:space="preserve">09/19/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F22">
@@ -1188,22 +1193,22 @@
       </c>
       <c t="inlineStr" r="G22">
         <is>
-          <t xml:space="preserve">RHG</t>
+          <t xml:space="preserve">Pway Lions</t>
         </is>
       </c>
       <c t="inlineStr" r="H22">
         <is>
+          <t xml:space="preserve">Aryans</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="I22">
+        <is>
+          <t xml:space="preserve">Pway Lions</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="J22">
+        <is>
           <t xml:space="preserve">11spartans</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="I22">
-        <is>
-          <t xml:space="preserve">11Spartans</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="J22">
-        <is>
-          <t xml:space="preserve">Nj Braves</t>
         </is>
       </c>
     </row>
@@ -1223,7 +1228,7 @@
       </c>
       <c t="inlineStr" r="E23">
         <is>
-          <t xml:space="preserve">09/12/2026</t>
+          <t xml:space="preserve">09/13/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F23">
@@ -1233,22 +1238,22 @@
       </c>
       <c t="inlineStr" r="G23">
         <is>
-          <t xml:space="preserve">Team Highlanders</t>
+          <t xml:space="preserve">PUNJAB XI</t>
         </is>
       </c>
       <c t="inlineStr" r="H23">
         <is>
-          <t xml:space="preserve">SAMP XI</t>
+          <t xml:space="preserve">Parsippany Phoenix XI</t>
         </is>
       </c>
       <c t="inlineStr" r="I23">
         <is>
-          <t xml:space="preserve">Team Highlanders</t>
+          <t xml:space="preserve">Parsippany Phoenix XI</t>
         </is>
       </c>
       <c t="inlineStr" r="J23">
         <is>
-          <t xml:space="preserve">Veerans</t>
+          <t xml:space="preserve">Falcons</t>
         </is>
       </c>
     </row>
@@ -1268,7 +1273,7 @@
       </c>
       <c t="inlineStr" r="E24">
         <is>
-          <t xml:space="preserve">09/12/2026</t>
+          <t xml:space="preserve">09/13/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F24">
@@ -1278,22 +1283,22 @@
       </c>
       <c t="inlineStr" r="G24">
         <is>
-          <t xml:space="preserve">Samudhra Gladiators</t>
+          <t xml:space="preserve">Blasters</t>
         </is>
       </c>
       <c t="inlineStr" r="H24">
         <is>
-          <t xml:space="preserve">Blue Aces CC</t>
+          <t xml:space="preserve">Edison Rebelz</t>
         </is>
       </c>
       <c t="inlineStr" r="I24">
         <is>
-          <t xml:space="preserve">Samudhra Gladiators</t>
+          <t xml:space="preserve">Edison Rebelz</t>
         </is>
       </c>
       <c t="inlineStr" r="J24">
         <is>
-          <t xml:space="preserve">Jersey Boys</t>
+          <t xml:space="preserve">Warriors</t>
         </is>
       </c>
     </row>
@@ -1313,7 +1318,7 @@
       </c>
       <c t="inlineStr" r="E25">
         <is>
-          <t xml:space="preserve">09/12/2026</t>
+          <t xml:space="preserve">09/13/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F25">
@@ -1323,22 +1328,22 @@
       </c>
       <c t="inlineStr" r="G25">
         <is>
-          <t xml:space="preserve">Gcc</t>
+          <t xml:space="preserve">Nj Braves</t>
         </is>
       </c>
       <c t="inlineStr" r="H25">
         <is>
-          <t xml:space="preserve">Maha CC</t>
+          <t xml:space="preserve">Veerans</t>
         </is>
       </c>
       <c t="inlineStr" r="I25">
         <is>
-          <t xml:space="preserve">GCC</t>
+          <t xml:space="preserve">Veerans</t>
         </is>
       </c>
       <c t="inlineStr" r="J25">
         <is>
-          <t xml:space="preserve">Nj Tigers</t>
+          <t xml:space="preserve">Youth For Sewa</t>
         </is>
       </c>
     </row>
@@ -1358,7 +1363,7 @@
       </c>
       <c t="inlineStr" r="E26">
         <is>
-          <t xml:space="preserve">09/12/2026</t>
+          <t xml:space="preserve">09/13/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F26">
@@ -1368,22 +1373,22 @@
       </c>
       <c t="inlineStr" r="G26">
         <is>
-          <t xml:space="preserve">Desi Warriors</t>
+          <t xml:space="preserve">Jersey Titans</t>
         </is>
       </c>
       <c t="inlineStr" r="H26">
         <is>
-          <t xml:space="preserve">Fdu Giants</t>
+          <t xml:space="preserve">Jersey Boys</t>
         </is>
       </c>
       <c t="inlineStr" r="I26">
         <is>
-          <t xml:space="preserve">Desi Warriors</t>
+          <t xml:space="preserve">Jersey Boys</t>
         </is>
       </c>
       <c t="inlineStr" r="J26">
         <is>
-          <t xml:space="preserve">Jetha 11</t>
+          <t xml:space="preserve">RHG</t>
         </is>
       </c>
     </row>
@@ -1403,7 +1408,7 @@
       </c>
       <c t="inlineStr" r="E27">
         <is>
-          <t xml:space="preserve">09/12/2026</t>
+          <t xml:space="preserve">09/13/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F27">
@@ -1413,22 +1418,22 @@
       </c>
       <c t="inlineStr" r="G27">
         <is>
-          <t xml:space="preserve">Sreeshti</t>
+          <t xml:space="preserve">Plainsboro Knights</t>
         </is>
       </c>
       <c t="inlineStr" r="H27">
         <is>
-          <t xml:space="preserve">Juggernaut</t>
+          <t xml:space="preserve">Nj Tigers</t>
         </is>
       </c>
       <c t="inlineStr" r="I27">
         <is>
-          <t xml:space="preserve">Sreeshti</t>
+          <t xml:space="preserve">NJ Tigers</t>
         </is>
       </c>
       <c t="inlineStr" r="J27">
         <is>
-          <t xml:space="preserve">Plainsboro Eagles</t>
+          <t xml:space="preserve">Team Highlanders</t>
         </is>
       </c>
     </row>
@@ -1448,7 +1453,7 @@
       </c>
       <c t="inlineStr" r="E28">
         <is>
-          <t xml:space="preserve">09/12/2026</t>
+          <t xml:space="preserve">09/13/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F28">
@@ -1458,22 +1463,22 @@
       </c>
       <c t="inlineStr" r="G28">
         <is>
-          <t xml:space="preserve">Hudson Hurricanes</t>
+          <t xml:space="preserve">Mercer Challengers</t>
         </is>
       </c>
       <c t="inlineStr" r="H28">
         <is>
-          <t xml:space="preserve">F5</t>
+          <t xml:space="preserve">Jetha 11</t>
         </is>
       </c>
       <c t="inlineStr" r="I28">
         <is>
-          <t xml:space="preserve">Hudson Hurricanes</t>
+          <t xml:space="preserve">Jetha 11</t>
         </is>
       </c>
       <c t="inlineStr" r="J28">
         <is>
-          <t xml:space="preserve">WCC</t>
+          <t xml:space="preserve">Samudhra Gladiators</t>
         </is>
       </c>
     </row>
@@ -1493,7 +1498,7 @@
       </c>
       <c t="inlineStr" r="E29">
         <is>
-          <t xml:space="preserve">09/12/2026</t>
+          <t xml:space="preserve">09/13/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F29">
@@ -1503,22 +1508,22 @@
       </c>
       <c t="inlineStr" r="G29">
         <is>
-          <t xml:space="preserve">Falcons</t>
+          <t xml:space="preserve">Storm Riders</t>
         </is>
       </c>
       <c t="inlineStr" r="H29">
         <is>
-          <t xml:space="preserve">Piscataway Avengers</t>
+          <t xml:space="preserve">Plainsboro Eagles</t>
         </is>
       </c>
       <c t="inlineStr" r="I29">
         <is>
-          <t xml:space="preserve">Falcons</t>
+          <t xml:space="preserve">Plainsboro Eagles</t>
         </is>
       </c>
       <c t="inlineStr" r="J29">
         <is>
-          <t xml:space="preserve">Aryans</t>
+          <t xml:space="preserve">Gcc</t>
         </is>
       </c>
     </row>
@@ -1538,7 +1543,7 @@
       </c>
       <c t="inlineStr" r="E30">
         <is>
-          <t xml:space="preserve">09/12/2026</t>
+          <t xml:space="preserve">09/13/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F30">
@@ -1548,22 +1553,22 @@
       </c>
       <c t="inlineStr" r="G30">
         <is>
-          <t xml:space="preserve">Warriors</t>
+          <t xml:space="preserve">Newport CC</t>
         </is>
       </c>
       <c t="inlineStr" r="H30">
         <is>
-          <t xml:space="preserve">Gryffindors</t>
+          <t xml:space="preserve">WCC</t>
         </is>
       </c>
       <c t="inlineStr" r="I30">
         <is>
-          <t xml:space="preserve">Warriors</t>
+          <t xml:space="preserve">WCC</t>
         </is>
       </c>
       <c t="inlineStr" r="J30">
         <is>
-          <t xml:space="preserve">Nj Stars CC</t>
+          <t xml:space="preserve">Desi Warriors</t>
         </is>
       </c>
     </row>
@@ -1583,7 +1588,7 @@
       </c>
       <c t="inlineStr" r="E31">
         <is>
-          <t xml:space="preserve">09/12/2026</t>
+          <t xml:space="preserve">09/13/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F31">
@@ -1593,22 +1598,22 @@
       </c>
       <c t="inlineStr" r="G31">
         <is>
-          <t xml:space="preserve">Youth For Sewa</t>
+          <t xml:space="preserve">Gujarat United XI</t>
         </is>
       </c>
       <c t="inlineStr" r="H31">
         <is>
-          <t xml:space="preserve">11spartans</t>
+          <t xml:space="preserve">Aryans</t>
         </is>
       </c>
       <c t="inlineStr" r="I31">
         <is>
-          <t xml:space="preserve">Youth For Sewa</t>
+          <t xml:space="preserve">Aryans</t>
         </is>
       </c>
       <c t="inlineStr" r="J31">
         <is>
-          <t xml:space="preserve">Parsippany Phoenix XI</t>
+          <t xml:space="preserve">Sreeshti</t>
         </is>
       </c>
     </row>
@@ -1628,7 +1633,7 @@
       </c>
       <c t="inlineStr" r="E32">
         <is>
-          <t xml:space="preserve">09/12/2026</t>
+          <t xml:space="preserve">09/13/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F32">
@@ -1638,22 +1643,22 @@
       </c>
       <c t="inlineStr" r="G32">
         <is>
-          <t xml:space="preserve">RHG</t>
+          <t xml:space="preserve">Pway Lions</t>
         </is>
       </c>
       <c t="inlineStr" r="H32">
         <is>
-          <t xml:space="preserve">Rowdy Rebels</t>
+          <t xml:space="preserve">Nj Stars CC</t>
         </is>
       </c>
       <c t="inlineStr" r="I32">
         <is>
-          <t xml:space="preserve">RHG</t>
+          <t xml:space="preserve">NJ Stars CC</t>
         </is>
       </c>
       <c t="inlineStr" r="J32">
         <is>
-          <t xml:space="preserve">Edison Rebelz</t>
+          <t xml:space="preserve">Hudson Hurricanes</t>
         </is>
       </c>
     </row>
@@ -1673,7 +1678,7 @@
       </c>
       <c t="inlineStr" r="E33">
         <is>
-          <t xml:space="preserve">09/13/2026</t>
+          <t xml:space="preserve">09/12/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F33">
@@ -1683,22 +1688,22 @@
       </c>
       <c t="inlineStr" r="G33">
         <is>
-          <t xml:space="preserve">Pway Lions</t>
+          <t xml:space="preserve">RHG</t>
         </is>
       </c>
       <c t="inlineStr" r="H33">
         <is>
-          <t xml:space="preserve">Nj Stars CC</t>
+          <t xml:space="preserve">Rowdy Rebels</t>
         </is>
       </c>
       <c t="inlineStr" r="I33">
         <is>
-          <t xml:space="preserve">NJ Stars CC</t>
+          <t xml:space="preserve">RHG</t>
         </is>
       </c>
       <c t="inlineStr" r="J33">
         <is>
-          <t xml:space="preserve">Hudson Hurricanes</t>
+          <t xml:space="preserve">Edison Rebelz</t>
         </is>
       </c>
     </row>
@@ -1718,7 +1723,7 @@
       </c>
       <c t="inlineStr" r="E34">
         <is>
-          <t xml:space="preserve">09/13/2026</t>
+          <t xml:space="preserve">09/12/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F34">
@@ -1728,22 +1733,22 @@
       </c>
       <c t="inlineStr" r="G34">
         <is>
-          <t xml:space="preserve">Gujarat United XI</t>
+          <t xml:space="preserve">Youth For Sewa</t>
         </is>
       </c>
       <c t="inlineStr" r="H34">
         <is>
-          <t xml:space="preserve">Aryans</t>
+          <t xml:space="preserve">11spartans</t>
         </is>
       </c>
       <c t="inlineStr" r="I34">
         <is>
-          <t xml:space="preserve">Aryans</t>
+          <t xml:space="preserve">Youth For Sewa</t>
         </is>
       </c>
       <c t="inlineStr" r="J34">
         <is>
-          <t xml:space="preserve">Sreeshti</t>
+          <t xml:space="preserve">Parsippany Phoenix XI</t>
         </is>
       </c>
     </row>
@@ -1763,7 +1768,7 @@
       </c>
       <c t="inlineStr" r="E35">
         <is>
-          <t xml:space="preserve">09/13/2026</t>
+          <t xml:space="preserve">09/12/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F35">
@@ -1773,22 +1778,17 @@
       </c>
       <c t="inlineStr" r="G35">
         <is>
-          <t xml:space="preserve">Newport CC</t>
+          <t xml:space="preserve">Warriors</t>
         </is>
       </c>
       <c t="inlineStr" r="H35">
         <is>
-          <t xml:space="preserve">WCC</t>
+          <t xml:space="preserve">Gryffindors</t>
         </is>
       </c>
       <c t="inlineStr" r="I35">
         <is>
-          <t xml:space="preserve">WCC</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="J35">
-        <is>
-          <t xml:space="preserve">Desi Warriors</t>
+          <t xml:space="preserve">Warriors</t>
         </is>
       </c>
     </row>
@@ -1808,7 +1808,7 @@
       </c>
       <c t="inlineStr" r="E36">
         <is>
-          <t xml:space="preserve">09/13/2026</t>
+          <t xml:space="preserve">09/12/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F36">
@@ -1818,22 +1818,22 @@
       </c>
       <c t="inlineStr" r="G36">
         <is>
-          <t xml:space="preserve">Storm Riders</t>
+          <t xml:space="preserve">Falcons</t>
         </is>
       </c>
       <c t="inlineStr" r="H36">
         <is>
-          <t xml:space="preserve">Plainsboro Eagles</t>
+          <t xml:space="preserve">Piscataway Avengers</t>
         </is>
       </c>
       <c t="inlineStr" r="I36">
         <is>
-          <t xml:space="preserve">Plainsboro Eagles</t>
+          <t xml:space="preserve">Falcons</t>
         </is>
       </c>
       <c t="inlineStr" r="J36">
         <is>
-          <t xml:space="preserve">Gcc</t>
+          <t xml:space="preserve">Aryans</t>
         </is>
       </c>
     </row>
@@ -1853,7 +1853,7 @@
       </c>
       <c t="inlineStr" r="E37">
         <is>
-          <t xml:space="preserve">09/13/2026</t>
+          <t xml:space="preserve">09/12/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F37">
@@ -1863,22 +1863,22 @@
       </c>
       <c t="inlineStr" r="G37">
         <is>
-          <t xml:space="preserve">Mercer Challengers</t>
+          <t xml:space="preserve">Hudson Hurricanes</t>
         </is>
       </c>
       <c t="inlineStr" r="H37">
         <is>
-          <t xml:space="preserve">Jetha 11</t>
+          <t xml:space="preserve">F5</t>
         </is>
       </c>
       <c t="inlineStr" r="I37">
         <is>
-          <t xml:space="preserve">Jetha 11</t>
+          <t xml:space="preserve">Hudson Hurricanes</t>
         </is>
       </c>
       <c t="inlineStr" r="J37">
         <is>
-          <t xml:space="preserve">Samudhra Gladiators</t>
+          <t xml:space="preserve">WCC</t>
         </is>
       </c>
     </row>
@@ -1898,7 +1898,7 @@
       </c>
       <c t="inlineStr" r="E38">
         <is>
-          <t xml:space="preserve">09/13/2026</t>
+          <t xml:space="preserve">09/12/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F38">
@@ -1908,22 +1908,22 @@
       </c>
       <c t="inlineStr" r="G38">
         <is>
-          <t xml:space="preserve">Plainsboro Knights</t>
+          <t xml:space="preserve">Sreeshti</t>
         </is>
       </c>
       <c t="inlineStr" r="H38">
         <is>
-          <t xml:space="preserve">Nj Tigers</t>
+          <t xml:space="preserve">Juggernaut</t>
         </is>
       </c>
       <c t="inlineStr" r="I38">
         <is>
-          <t xml:space="preserve">NJ Tigers</t>
+          <t xml:space="preserve">Sreeshti</t>
         </is>
       </c>
       <c t="inlineStr" r="J38">
         <is>
-          <t xml:space="preserve">Team Highlanders</t>
+          <t xml:space="preserve">Plainsboro Eagles</t>
         </is>
       </c>
     </row>
@@ -1943,7 +1943,7 @@
       </c>
       <c t="inlineStr" r="E39">
         <is>
-          <t xml:space="preserve">09/13/2026</t>
+          <t xml:space="preserve">09/12/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F39">
@@ -1953,22 +1953,22 @@
       </c>
       <c t="inlineStr" r="G39">
         <is>
-          <t xml:space="preserve">Jersey Titans</t>
+          <t xml:space="preserve">Desi Warriors</t>
         </is>
       </c>
       <c t="inlineStr" r="H39">
         <is>
-          <t xml:space="preserve">Jersey Boys</t>
+          <t xml:space="preserve">Fdu Giants</t>
         </is>
       </c>
       <c t="inlineStr" r="I39">
         <is>
-          <t xml:space="preserve">Jersey Boys</t>
+          <t xml:space="preserve">Desi Warriors</t>
         </is>
       </c>
       <c t="inlineStr" r="J39">
         <is>
-          <t xml:space="preserve">RHG</t>
+          <t xml:space="preserve">Jetha 11</t>
         </is>
       </c>
     </row>
@@ -1988,7 +1988,7 @@
       </c>
       <c t="inlineStr" r="E40">
         <is>
-          <t xml:space="preserve">09/13/2026</t>
+          <t xml:space="preserve">09/12/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F40">
@@ -1998,22 +1998,22 @@
       </c>
       <c t="inlineStr" r="G40">
         <is>
-          <t xml:space="preserve">Nj Braves</t>
+          <t xml:space="preserve">Gcc</t>
         </is>
       </c>
       <c t="inlineStr" r="H40">
         <is>
-          <t xml:space="preserve">Veerans</t>
+          <t xml:space="preserve">Maha CC</t>
         </is>
       </c>
       <c t="inlineStr" r="I40">
         <is>
-          <t xml:space="preserve">Veerans</t>
+          <t xml:space="preserve">GCC</t>
         </is>
       </c>
       <c t="inlineStr" r="J40">
         <is>
-          <t xml:space="preserve">Youth For Sewa</t>
+          <t xml:space="preserve">Nj Tigers</t>
         </is>
       </c>
     </row>
@@ -2033,7 +2033,7 @@
       </c>
       <c t="inlineStr" r="E41">
         <is>
-          <t xml:space="preserve">09/13/2026</t>
+          <t xml:space="preserve">09/12/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F41">
@@ -2043,22 +2043,22 @@
       </c>
       <c t="inlineStr" r="G41">
         <is>
-          <t xml:space="preserve">Blasters</t>
+          <t xml:space="preserve">Samudhra Gladiators</t>
         </is>
       </c>
       <c t="inlineStr" r="H41">
         <is>
-          <t xml:space="preserve">Edison Rebelz</t>
+          <t xml:space="preserve">Blue Aces CC</t>
         </is>
       </c>
       <c t="inlineStr" r="I41">
         <is>
-          <t xml:space="preserve">Edison Rebelz</t>
+          <t xml:space="preserve">Samudhra Gladiators</t>
         </is>
       </c>
       <c t="inlineStr" r="J41">
         <is>
-          <t xml:space="preserve">Warriors</t>
+          <t xml:space="preserve">Jersey Boys</t>
         </is>
       </c>
     </row>
@@ -2078,7 +2078,7 @@
       </c>
       <c t="inlineStr" r="E42">
         <is>
-          <t xml:space="preserve">09/13/2026</t>
+          <t xml:space="preserve">09/12/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F42">
@@ -2088,22 +2088,22 @@
       </c>
       <c t="inlineStr" r="G42">
         <is>
-          <t xml:space="preserve">PUNJAB XI</t>
+          <t xml:space="preserve">Team Highlanders</t>
         </is>
       </c>
       <c t="inlineStr" r="H42">
         <is>
-          <t xml:space="preserve">Parsippany Phoenix XI</t>
+          <t xml:space="preserve">SAMP XI</t>
         </is>
       </c>
       <c t="inlineStr" r="I42">
         <is>
-          <t xml:space="preserve">Parsippany Phoenix XI</t>
+          <t xml:space="preserve">Team Highlanders</t>
         </is>
       </c>
       <c t="inlineStr" r="J42">
         <is>
-          <t xml:space="preserve">Falcons</t>
+          <t xml:space="preserve">Veerans</t>
         </is>
       </c>
     </row>
@@ -2123,7 +2123,7 @@
       </c>
       <c t="inlineStr" r="E43">
         <is>
-          <t xml:space="preserve">09/19/2026</t>
+          <t xml:space="preserve">08/30/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F43">
@@ -2133,22 +2133,22 @@
       </c>
       <c t="inlineStr" r="G43">
         <is>
-          <t xml:space="preserve">Pway Lions</t>
+          <t xml:space="preserve">RHG</t>
         </is>
       </c>
       <c t="inlineStr" r="H43">
         <is>
-          <t xml:space="preserve">Aryans</t>
+          <t xml:space="preserve">11spartans</t>
         </is>
       </c>
       <c t="inlineStr" r="I43">
         <is>
-          <t xml:space="preserve">Pway Lions</t>
+          <t xml:space="preserve">11Spartans</t>
         </is>
       </c>
       <c t="inlineStr" r="J43">
         <is>
-          <t xml:space="preserve">11spartans</t>
+          <t xml:space="preserve">Nj Braves</t>
         </is>
       </c>
     </row>
@@ -2168,7 +2168,7 @@
       </c>
       <c t="inlineStr" r="E44">
         <is>
-          <t xml:space="preserve">09/19/2026</t>
+          <t xml:space="preserve">08/30/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F44">
@@ -2178,22 +2178,22 @@
       </c>
       <c t="inlineStr" r="G44">
         <is>
-          <t xml:space="preserve">Gujarat United XI</t>
+          <t xml:space="preserve">Youth For Sewa</t>
         </is>
       </c>
       <c t="inlineStr" r="H44">
         <is>
-          <t xml:space="preserve">WCC</t>
+          <t xml:space="preserve">Gryffindors</t>
         </is>
       </c>
       <c t="inlineStr" r="I44">
         <is>
-          <t xml:space="preserve">Gujarat United XI</t>
+          <t xml:space="preserve">Gryffindors</t>
         </is>
       </c>
       <c t="inlineStr" r="J44">
         <is>
-          <t xml:space="preserve">Gryffindors</t>
+          <t xml:space="preserve">Blasters</t>
         </is>
       </c>
     </row>
@@ -2213,7 +2213,7 @@
       </c>
       <c t="inlineStr" r="E45">
         <is>
-          <t xml:space="preserve">09/19/2026</t>
+          <t xml:space="preserve">08/30/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F45">
@@ -2223,22 +2223,22 @@
       </c>
       <c t="inlineStr" r="G45">
         <is>
-          <t xml:space="preserve">Newport CC</t>
+          <t xml:space="preserve">Warriors</t>
         </is>
       </c>
       <c t="inlineStr" r="H45">
         <is>
-          <t xml:space="preserve">Plainsboro Eagles</t>
+          <t xml:space="preserve">Piscataway Avengers</t>
         </is>
       </c>
       <c t="inlineStr" r="I45">
         <is>
-          <t xml:space="preserve">Newport CC</t>
+          <t xml:space="preserve">Piscataway Avengers</t>
         </is>
       </c>
       <c t="inlineStr" r="J45">
         <is>
-          <t xml:space="preserve">Piscataway Avengers</t>
+          <t xml:space="preserve">PUNJAB XI</t>
         </is>
       </c>
     </row>
@@ -2258,7 +2258,7 @@
       </c>
       <c t="inlineStr" r="E46">
         <is>
-          <t xml:space="preserve">09/19/2026</t>
+          <t xml:space="preserve">08/30/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F46">
@@ -2268,22 +2268,22 @@
       </c>
       <c t="inlineStr" r="G46">
         <is>
-          <t xml:space="preserve">Storm Riders</t>
+          <t xml:space="preserve">Falcons</t>
         </is>
       </c>
       <c t="inlineStr" r="H46">
         <is>
-          <t xml:space="preserve">Jetha 11</t>
+          <t xml:space="preserve">F5</t>
         </is>
       </c>
       <c t="inlineStr" r="I46">
         <is>
-          <t xml:space="preserve">Storm Riders</t>
+          <t xml:space="preserve">F5</t>
         </is>
       </c>
       <c t="inlineStr" r="J46">
         <is>
-          <t xml:space="preserve">F5</t>
+          <t xml:space="preserve">Pway Lions</t>
         </is>
       </c>
     </row>
@@ -2303,7 +2303,7 @@
       </c>
       <c t="inlineStr" r="E47">
         <is>
-          <t xml:space="preserve">09/19/2026</t>
+          <t xml:space="preserve">08/30/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F47">
@@ -2313,22 +2313,22 @@
       </c>
       <c t="inlineStr" r="G47">
         <is>
-          <t xml:space="preserve">Mercer Challengers</t>
+          <t xml:space="preserve">Hudson Hurricanes</t>
         </is>
       </c>
       <c t="inlineStr" r="H47">
         <is>
-          <t xml:space="preserve">Nj Tigers</t>
+          <t xml:space="preserve">Juggernaut</t>
         </is>
       </c>
       <c t="inlineStr" r="I47">
         <is>
-          <t xml:space="preserve">Mercer Challengers</t>
+          <t xml:space="preserve">Juggernaut</t>
         </is>
       </c>
       <c t="inlineStr" r="J47">
         <is>
-          <t xml:space="preserve">Juggernaut</t>
+          <t xml:space="preserve">Gujarat United XI</t>
         </is>
       </c>
     </row>
@@ -2348,7 +2348,7 @@
       </c>
       <c t="inlineStr" r="E48">
         <is>
-          <t xml:space="preserve">09/19/2026</t>
+          <t xml:space="preserve">08/30/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F48">
@@ -2358,22 +2358,22 @@
       </c>
       <c t="inlineStr" r="G48">
         <is>
-          <t xml:space="preserve">Plainsboro Knights</t>
+          <t xml:space="preserve">Sreeshti</t>
         </is>
       </c>
       <c t="inlineStr" r="H48">
         <is>
-          <t xml:space="preserve">Jersey Boys</t>
+          <t xml:space="preserve">Fdu Giants</t>
         </is>
       </c>
       <c t="inlineStr" r="I48">
         <is>
-          <t xml:space="preserve">Plainsboro Knights</t>
+          <t xml:space="preserve">FDU Giants</t>
         </is>
       </c>
       <c t="inlineStr" r="J48">
         <is>
-          <t xml:space="preserve">Fdu Giants</t>
+          <t xml:space="preserve">Newport CC</t>
         </is>
       </c>
     </row>
@@ -2393,7 +2393,7 @@
       </c>
       <c t="inlineStr" r="E49">
         <is>
-          <t xml:space="preserve">09/19/2026</t>
+          <t xml:space="preserve">08/30/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F49">
@@ -2403,22 +2403,22 @@
       </c>
       <c t="inlineStr" r="G49">
         <is>
-          <t xml:space="preserve">Jersey Titans</t>
+          <t xml:space="preserve">Desi Warriors</t>
         </is>
       </c>
       <c t="inlineStr" r="H49">
         <is>
-          <t xml:space="preserve">Veerans</t>
+          <t xml:space="preserve">Maha CC</t>
         </is>
       </c>
       <c t="inlineStr" r="I49">
         <is>
-          <t xml:space="preserve">Jersey Titans</t>
+          <t xml:space="preserve">Maha CC</t>
         </is>
       </c>
       <c t="inlineStr" r="J49">
         <is>
-          <t xml:space="preserve">Maha CC</t>
+          <t xml:space="preserve">Storm Riders</t>
         </is>
       </c>
     </row>
@@ -2438,7 +2438,7 @@
       </c>
       <c t="inlineStr" r="E50">
         <is>
-          <t xml:space="preserve">09/19/2026</t>
+          <t xml:space="preserve">08/30/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F50">
@@ -2448,22 +2448,22 @@
       </c>
       <c t="inlineStr" r="G50">
         <is>
-          <t xml:space="preserve">Nj Braves</t>
+          <t xml:space="preserve">Gcc</t>
         </is>
       </c>
       <c t="inlineStr" r="H50">
         <is>
-          <t xml:space="preserve">Edison Rebelz</t>
+          <t xml:space="preserve">Blue Aces CC</t>
         </is>
       </c>
       <c t="inlineStr" r="I50">
         <is>
-          <t xml:space="preserve">NJ Braves</t>
+          <t xml:space="preserve">Blue Aces CC</t>
         </is>
       </c>
       <c t="inlineStr" r="J50">
         <is>
-          <t xml:space="preserve">Blue Aces CC</t>
+          <t xml:space="preserve">Mercer Challengers</t>
         </is>
       </c>
     </row>
@@ -2483,7 +2483,7 @@
       </c>
       <c t="inlineStr" r="E51">
         <is>
-          <t xml:space="preserve">09/19/2026</t>
+          <t xml:space="preserve">08/30/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F51">
@@ -2493,22 +2493,22 @@
       </c>
       <c t="inlineStr" r="G51">
         <is>
-          <t xml:space="preserve">Blasters</t>
+          <t xml:space="preserve">Samudhra Gladiators</t>
         </is>
       </c>
       <c t="inlineStr" r="H51">
         <is>
-          <t xml:space="preserve">Parsippany Phoenix XI</t>
+          <t xml:space="preserve">SAMP XI</t>
         </is>
       </c>
       <c t="inlineStr" r="I51">
         <is>
-          <t xml:space="preserve">Blasters</t>
+          <t xml:space="preserve">Samp XI</t>
         </is>
       </c>
       <c t="inlineStr" r="J51">
         <is>
-          <t xml:space="preserve">SAMP XI</t>
+          <t xml:space="preserve">Plainsboro Knights</t>
         </is>
       </c>
     </row>
@@ -2528,7 +2528,7 @@
       </c>
       <c t="inlineStr" r="E52">
         <is>
-          <t xml:space="preserve">09/19/2026</t>
+          <t xml:space="preserve">08/30/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F52">
@@ -2538,22 +2538,22 @@
       </c>
       <c t="inlineStr" r="G52">
         <is>
-          <t xml:space="preserve">PUNJAB XI</t>
+          <t xml:space="preserve">Team Highlanders</t>
         </is>
       </c>
       <c t="inlineStr" r="H52">
         <is>
-          <t xml:space="preserve">Nj Stars CC</t>
+          <t xml:space="preserve">Rowdy Rebels</t>
         </is>
       </c>
       <c t="inlineStr" r="I52">
         <is>
-          <t xml:space="preserve">Punjab XI</t>
+          <t xml:space="preserve">Rowdy Rebels</t>
         </is>
       </c>
       <c t="inlineStr" r="J52">
         <is>
-          <t xml:space="preserve">Rowdy Rebels</t>
+          <t xml:space="preserve">Jersey Titans</t>
         </is>
       </c>
     </row>
@@ -2573,7 +2573,7 @@
       </c>
       <c t="inlineStr" r="E53">
         <is>
-          <t xml:space="preserve">09/20/2026</t>
+          <t xml:space="preserve">08/29/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F53">
@@ -2583,22 +2583,22 @@
       </c>
       <c t="inlineStr" r="G53">
         <is>
-          <t xml:space="preserve">Team Highlanders</t>
+          <t xml:space="preserve">PUNJAB XI</t>
         </is>
       </c>
       <c t="inlineStr" r="H53">
         <is>
-          <t xml:space="preserve">Blue Aces CC</t>
+          <t xml:space="preserve">Edison Rebelz</t>
         </is>
       </c>
       <c t="inlineStr" r="I53">
         <is>
-          <t xml:space="preserve">Blue Aces CC</t>
+          <t xml:space="preserve">Punjab XI</t>
         </is>
       </c>
       <c t="inlineStr" r="J53">
         <is>
-          <t xml:space="preserve">Plainsboro Knights</t>
+          <t xml:space="preserve">SAMP XI</t>
         </is>
       </c>
     </row>
@@ -2618,7 +2618,7 @@
       </c>
       <c t="inlineStr" r="E54">
         <is>
-          <t xml:space="preserve">09/20/2026</t>
+          <t xml:space="preserve">08/29/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F54">
@@ -2628,22 +2628,22 @@
       </c>
       <c t="inlineStr" r="G54">
         <is>
-          <t xml:space="preserve">Samudhra Gladiators</t>
+          <t xml:space="preserve">Blasters</t>
         </is>
       </c>
       <c t="inlineStr" r="H54">
         <is>
-          <t xml:space="preserve">Maha CC</t>
+          <t xml:space="preserve">Veerans</t>
         </is>
       </c>
       <c t="inlineStr" r="I54">
         <is>
-          <t xml:space="preserve">Maha CC</t>
+          <t xml:space="preserve">Blasters</t>
         </is>
       </c>
       <c t="inlineStr" r="J54">
         <is>
-          <t xml:space="preserve">Mercer Challengers</t>
+          <t xml:space="preserve">Blue Aces CC</t>
         </is>
       </c>
     </row>
@@ -2663,7 +2663,7 @@
       </c>
       <c t="inlineStr" r="E55">
         <is>
-          <t xml:space="preserve">09/20/2026</t>
+          <t xml:space="preserve">08/29/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F55">
@@ -2673,22 +2673,22 @@
       </c>
       <c t="inlineStr" r="G55">
         <is>
-          <t xml:space="preserve">Gcc</t>
+          <t xml:space="preserve">Nj Braves</t>
         </is>
       </c>
       <c t="inlineStr" r="H55">
         <is>
-          <t xml:space="preserve">Fdu Giants</t>
+          <t xml:space="preserve">Jersey Boys</t>
         </is>
       </c>
       <c t="inlineStr" r="I55">
         <is>
-          <t xml:space="preserve">FDU Giants</t>
+          <t xml:space="preserve">NJ Braves</t>
         </is>
       </c>
       <c t="inlineStr" r="J55">
         <is>
-          <t xml:space="preserve">Storm Riders</t>
+          <t xml:space="preserve">Maha CC</t>
         </is>
       </c>
     </row>
@@ -2708,7 +2708,7 @@
       </c>
       <c t="inlineStr" r="E56">
         <is>
-          <t xml:space="preserve">09/20/2026</t>
+          <t xml:space="preserve">08/29/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F56">
@@ -2718,22 +2718,22 @@
       </c>
       <c t="inlineStr" r="G56">
         <is>
-          <t xml:space="preserve">Desi Warriors</t>
+          <t xml:space="preserve">Jersey Titans</t>
         </is>
       </c>
       <c t="inlineStr" r="H56">
         <is>
-          <t xml:space="preserve">Juggernaut</t>
+          <t xml:space="preserve">Nj Tigers</t>
         </is>
       </c>
       <c t="inlineStr" r="I56">
         <is>
-          <t xml:space="preserve">Juggernaut</t>
+          <t xml:space="preserve">Jersey Titans</t>
         </is>
       </c>
       <c t="inlineStr" r="J56">
         <is>
-          <t xml:space="preserve">Newport CC</t>
+          <t xml:space="preserve">Fdu Giants</t>
         </is>
       </c>
     </row>
@@ -2753,7 +2753,7 @@
       </c>
       <c t="inlineStr" r="E57">
         <is>
-          <t xml:space="preserve">09/20/2026</t>
+          <t xml:space="preserve">08/29/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F57">
@@ -2763,22 +2763,22 @@
       </c>
       <c t="inlineStr" r="G57">
         <is>
-          <t xml:space="preserve">Sreeshti</t>
+          <t xml:space="preserve">Plainsboro Knights</t>
         </is>
       </c>
       <c t="inlineStr" r="H57">
         <is>
-          <t xml:space="preserve">F5</t>
+          <t xml:space="preserve">Jetha 11</t>
         </is>
       </c>
       <c t="inlineStr" r="I57">
         <is>
-          <t xml:space="preserve">F5</t>
+          <t xml:space="preserve">Plainsboro Knights</t>
         </is>
       </c>
       <c t="inlineStr" r="J57">
         <is>
-          <t xml:space="preserve">Gujarat United XI</t>
+          <t xml:space="preserve">Juggernaut</t>
         </is>
       </c>
     </row>
@@ -2798,7 +2798,7 @@
       </c>
       <c t="inlineStr" r="E58">
         <is>
-          <t xml:space="preserve">09/20/2026</t>
+          <t xml:space="preserve">08/29/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F58">
@@ -2808,22 +2808,22 @@
       </c>
       <c t="inlineStr" r="G58">
         <is>
-          <t xml:space="preserve">Hudson Hurricanes</t>
+          <t xml:space="preserve">Mercer Challengers</t>
         </is>
       </c>
       <c t="inlineStr" r="H58">
         <is>
-          <t xml:space="preserve">Piscataway Avengers</t>
+          <t xml:space="preserve">Plainsboro Eagles</t>
         </is>
       </c>
       <c t="inlineStr" r="I58">
         <is>
-          <t xml:space="preserve">Piscataway Avengers</t>
+          <t xml:space="preserve">Mercer Challengers</t>
         </is>
       </c>
       <c t="inlineStr" r="J58">
         <is>
-          <t xml:space="preserve">Pway Lions</t>
+          <t xml:space="preserve">F5</t>
         </is>
       </c>
     </row>
@@ -2843,7 +2843,7 @@
       </c>
       <c t="inlineStr" r="E59">
         <is>
-          <t xml:space="preserve">09/20/2026</t>
+          <t xml:space="preserve">08/29/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F59">
@@ -2853,22 +2853,22 @@
       </c>
       <c t="inlineStr" r="G59">
         <is>
-          <t xml:space="preserve">Falcons</t>
+          <t xml:space="preserve">Storm Riders</t>
         </is>
       </c>
       <c t="inlineStr" r="H59">
         <is>
-          <t xml:space="preserve">Gryffindors</t>
+          <t xml:space="preserve">WCC</t>
         </is>
       </c>
       <c t="inlineStr" r="I59">
         <is>
-          <t xml:space="preserve">Gryffindors</t>
+          <t xml:space="preserve">Storm Riders</t>
         </is>
       </c>
       <c t="inlineStr" r="J59">
         <is>
-          <t xml:space="preserve">PUNJAB XI</t>
+          <t xml:space="preserve">Piscataway Avengers</t>
         </is>
       </c>
     </row>
@@ -2888,7 +2888,7 @@
       </c>
       <c t="inlineStr" r="E60">
         <is>
-          <t xml:space="preserve">09/20/2026</t>
+          <t xml:space="preserve">08/29/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F60">
@@ -2898,22 +2898,22 @@
       </c>
       <c t="inlineStr" r="G60">
         <is>
-          <t xml:space="preserve">Warriors</t>
+          <t xml:space="preserve">Newport CC</t>
         </is>
       </c>
       <c t="inlineStr" r="H60">
         <is>
-          <t xml:space="preserve">11spartans</t>
+          <t xml:space="preserve">Aryans</t>
         </is>
       </c>
       <c t="inlineStr" r="I60">
         <is>
-          <t xml:space="preserve">11Spartans</t>
+          <t xml:space="preserve">Newport CC</t>
         </is>
       </c>
       <c t="inlineStr" r="J60">
         <is>
-          <t xml:space="preserve">Blasters</t>
+          <t xml:space="preserve">Gryffindors</t>
         </is>
       </c>
     </row>
@@ -2933,7 +2933,7 @@
       </c>
       <c t="inlineStr" r="E61">
         <is>
-          <t xml:space="preserve">09/20/2026</t>
+          <t xml:space="preserve">08/29/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F61">
@@ -2943,22 +2943,22 @@
       </c>
       <c t="inlineStr" r="G61">
         <is>
-          <t xml:space="preserve">Youth For Sewa</t>
+          <t xml:space="preserve">Gujarat United XI</t>
         </is>
       </c>
       <c t="inlineStr" r="H61">
         <is>
-          <t xml:space="preserve">Rowdy Rebels</t>
+          <t xml:space="preserve">Nj Stars CC</t>
         </is>
       </c>
       <c t="inlineStr" r="I61">
         <is>
-          <t xml:space="preserve">Rowdy Rebels</t>
+          <t xml:space="preserve">Gujarat United XI</t>
         </is>
       </c>
       <c t="inlineStr" r="J61">
         <is>
-          <t xml:space="preserve">Nj Braves</t>
+          <t xml:space="preserve">11spartans</t>
         </is>
       </c>
     </row>
@@ -2978,7 +2978,7 @@
       </c>
       <c t="inlineStr" r="E62">
         <is>
-          <t xml:space="preserve">09/20/2026</t>
+          <t xml:space="preserve">08/29/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F62">
@@ -2988,22 +2988,22 @@
       </c>
       <c t="inlineStr" r="G62">
         <is>
-          <t xml:space="preserve">RHG</t>
+          <t xml:space="preserve">Pway Lions</t>
         </is>
       </c>
       <c t="inlineStr" r="H62">
         <is>
-          <t xml:space="preserve">SAMP XI</t>
+          <t xml:space="preserve">Parsippany Phoenix XI</t>
         </is>
       </c>
       <c t="inlineStr" r="I62">
         <is>
-          <t xml:space="preserve">Samp XI</t>
+          <t xml:space="preserve">Pway Lions</t>
         </is>
       </c>
       <c t="inlineStr" r="J62">
         <is>
-          <t xml:space="preserve">Jersey Titans</t>
+          <t xml:space="preserve">Rowdy Rebels</t>
         </is>
       </c>
     </row>

</xml_diff>